<commit_message>
feature:- create youth club - work in progress
</commit_message>
<xml_diff>
--- a/resources/Youth_prod.xlsx
+++ b/resources/Youth_prod.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>Email</t>
   </si>
@@ -96,6 +96,12 @@
   </si>
   <si>
     <t>EldonTrantow@yopmail.com</t>
+  </si>
+  <si>
+    <t>VeolaConsidine@yopmail.com</t>
+  </si>
+  <si>
+    <t>YvoneBerge@yopmail.com</t>
   </si>
 </sst>
 </file>
@@ -1255,7 +1261,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <sheetData>
     <row r="1" spans="1:1">
@@ -1373,6 +1379,16 @@
         <v>22</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="s" s="0">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s" s="0">
+        <v>24</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>

<commit_message>
feat: add youth Basic Info fill + Experiential Learning navigation + Opportunity near me flow
</commit_message>
<xml_diff>
--- a/resources/Youth_prod.xlsx
+++ b/resources/Youth_prod.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Email</t>
   </si>
@@ -96,6 +96,9 @@
   </si>
   <si>
     <t>EldonTrantow@yopmail.com</t>
+  </si>
+  <si>
+    <t>TwylaBosco@yopmail.com</t>
   </si>
 </sst>
 </file>
@@ -1255,7 +1258,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <sheetData>
     <row r="1" spans="1:1">
@@ -1373,6 +1376,11 @@
         <v>22</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="s" s="0">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>

<commit_message>
feat: blog module - create blog, verify pending status, add to all-modules + workflows
</commit_message>
<xml_diff>
--- a/resources/Youth_prod.xlsx
+++ b/resources/Youth_prod.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>Email</t>
   </si>
@@ -96,6 +96,24 @@
   </si>
   <si>
     <t>EldonTrantow@yopmail.com</t>
+  </si>
+  <si>
+    <t>RhiannonWitting@yopmail.com</t>
+  </si>
+  <si>
+    <t>ReidDoyle@yopmail.com</t>
+  </si>
+  <si>
+    <t>MarlinHellerJr@yopmail.com</t>
+  </si>
+  <si>
+    <t>BurtonBatz@yopmail.com</t>
+  </si>
+  <si>
+    <t>BradRyan@yopmail.com</t>
+  </si>
+  <si>
+    <t>AllegraMcClure@yopmail.com</t>
   </si>
 </sst>
 </file>
@@ -1255,7 +1273,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <sheetData>
     <row r="1" spans="1:1">
@@ -1373,6 +1391,36 @@
         <v>22</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="s" s="0">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s" s="0">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s" s="0">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s" s="0">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>

<commit_message>
fix: replace Yopmail with Maildrop API for OTP — eliminates CI flakiness - RegistrationPage: email changed from @yopmail.com to @maildrop.cc - RegistrationPage: fetchAndVerifyOTP() now uses Maildrop GraphQL API (no browser tab) - LoginPage: fetchOTPFromYopmail() rewritten to use Maildrop API - No more Yopmail popup/ad/iframe issues on CI - Tested locally: registration passes in 62s with API-based OTP
</commit_message>
<xml_diff>
--- a/resources/Youth_prod.xlsx
+++ b/resources/Youth_prod.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="40">
   <si>
     <t>yco71304@maildrop.cc</t>
   </si>
@@ -131,6 +131,9 @@
   </si>
   <si>
     <t>Nai Disha Enclave Beta Youth Club</t>
+  </si>
+  <si>
+    <t>TheronMurazik@maildrop.cc</t>
   </si>
 </sst>
 </file>
@@ -1351,7 +1354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A28"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="16.8"/>
   <sheetData>
     <row r="1">
@@ -1544,6 +1547,11 @@
     <row r="28">
       <c r="A28" t="s" s="0">
         <v>10</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s" s="0">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Registration + Logout + Login test with hourly GitHub Actions workflow (Yopmail OTP)
</commit_message>
<xml_diff>
--- a/resources/Youth_prod.xlsx
+++ b/resources/Youth_prod.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="42">
   <si>
     <t>yco71304@maildrop.cc</t>
   </si>
@@ -134,6 +134,12 @@
   </si>
   <si>
     <t>TheronMurazik@maildrop.cc</t>
+  </si>
+  <si>
+    <t>vincestiedemann@yopmail.com</t>
+  </si>
+  <si>
+    <t>hermandouglasjr@yopmail.com</t>
   </si>
 </sst>
 </file>
@@ -1354,7 +1360,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A31"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="16.8"/>
   <sheetData>
     <row r="1">
@@ -1552,6 +1558,16 @@
     <row r="29">
       <c r="A29" t="s" s="0">
         <v>39</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s" s="0">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s" s="0">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix: Registration OTP regex to match only 6-digit codes (not years)
</commit_message>
<xml_diff>
--- a/resources/Youth_prod.xlsx
+++ b/resources/Youth_prod.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="43">
   <si>
     <t>yco71304@maildrop.cc</t>
   </si>
@@ -140,6 +140,9 @@
   </si>
   <si>
     <t>hermandouglasjr@yopmail.com</t>
+  </si>
+  <si>
+    <t>msquentinwisozk@yopmail.com</t>
   </si>
 </sst>
 </file>
@@ -1360,7 +1363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A31"/>
+  <dimension ref="A1:A32"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="16.8"/>
   <sheetData>
     <row r="1">
@@ -1568,6 +1571,11 @@
     <row r="31">
       <c r="A31" t="s" s="0">
         <v>41</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s" s="0">
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>